<commit_message>
captura 2026-10-31 19:31 UTC
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -750,7 +750,7 @@
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
@@ -860,7 +860,7 @@
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE3" s="2" t="inlineStr">
@@ -966,7 +966,7 @@
       </c>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE4" s="2" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE5" s="2" t="inlineStr">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
@@ -1276,7 +1276,7 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="AD8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE8" s="2" t="inlineStr">
@@ -1484,7 +1484,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -1586,7 +1586,7 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
@@ -1688,7 +1688,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -1794,7 +1794,7 @@
       </c>
       <c r="AD12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE12" s="2" t="inlineStr">
@@ -1900,7 +1900,7 @@
       </c>
       <c r="AD13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE13" s="2" t="inlineStr">
@@ -2006,7 +2006,7 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE14" s="2" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE15" s="2" t="inlineStr">
@@ -2214,7 +2214,7 @@
       </c>
       <c r="AD16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE16" s="2" t="inlineStr">
@@ -2316,7 +2316,7 @@
       </c>
       <c r="AD17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE17" s="2" t="inlineStr">
@@ -2422,7 +2422,7 @@
       </c>
       <c r="AD18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE18" s="2" t="inlineStr">
@@ -2528,7 +2528,7 @@
       </c>
       <c r="AD19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE19" s="2" t="inlineStr">
@@ -2634,7 +2634,7 @@
       </c>
       <c r="AD20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE20" s="2" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="AD21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE21" s="2" t="inlineStr">
@@ -2842,7 +2842,7 @@
       </c>
       <c r="AD22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE22" s="2" t="inlineStr">
@@ -2944,7 +2944,7 @@
       </c>
       <c r="AD23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE23" s="2" t="inlineStr">
@@ -3046,7 +3046,7 @@
       </c>
       <c r="AD24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE24" s="2" t="inlineStr">
@@ -3148,7 +3148,7 @@
       </c>
       <c r="AD25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE25" s="2" t="inlineStr">
@@ -3250,7 +3250,7 @@
       </c>
       <c r="AD26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE26" s="2" t="inlineStr">
@@ -3352,7 +3352,7 @@
       </c>
       <c r="AD27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE27" s="2" t="inlineStr">
@@ -3454,7 +3454,7 @@
       </c>
       <c r="AD28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE28" s="2" t="inlineStr">
@@ -3560,7 +3560,7 @@
       </c>
       <c r="AD29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE29" s="2" t="inlineStr">
@@ -3662,7 +3662,7 @@
       </c>
       <c r="AD30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE30" s="2" t="inlineStr">
@@ -3768,7 +3768,7 @@
       </c>
       <c r="AD31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE31" s="2" t="inlineStr">
@@ -3870,7 +3870,7 @@
       </c>
       <c r="AD32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE32" s="2" t="inlineStr">
@@ -3976,7 +3976,7 @@
       </c>
       <c r="AD33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE33" s="2" t="inlineStr">
@@ -4078,7 +4078,7 @@
       </c>
       <c r="AD34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE34" s="2" t="inlineStr">
@@ -4184,7 +4184,7 @@
       </c>
       <c r="AD35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE35" s="2" t="inlineStr">
@@ -4290,7 +4290,7 @@
       </c>
       <c r="AD36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE36" s="2" t="inlineStr">
@@ -4392,7 +4392,7 @@
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE37" s="2" t="inlineStr">
@@ -4498,7 +4498,7 @@
       </c>
       <c r="AD38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE38" s="2" t="inlineStr">
@@ -4604,7 +4604,7 @@
       </c>
       <c r="AD39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE39" s="2" t="inlineStr">
@@ -4710,7 +4710,7 @@
       </c>
       <c r="AD40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE40" s="2" t="inlineStr">
@@ -4816,7 +4816,7 @@
       </c>
       <c r="AD41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE41" s="2" t="inlineStr">
@@ -4922,7 +4922,7 @@
       </c>
       <c r="AD42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE42" s="2" t="inlineStr">
@@ -5028,7 +5028,7 @@
       </c>
       <c r="AD43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE43" s="2" t="inlineStr">
@@ -5134,7 +5134,7 @@
       </c>
       <c r="AD44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE44" s="2" t="inlineStr">
@@ -5240,7 +5240,7 @@
       </c>
       <c r="AD45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE45" s="2" t="inlineStr">
@@ -5346,7 +5346,7 @@
       </c>
       <c r="AD46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE46" s="2" t="inlineStr">
@@ -5452,7 +5452,7 @@
       </c>
       <c r="AD47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE47" s="2" t="inlineStr">
@@ -5558,7 +5558,7 @@
       </c>
       <c r="AD48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE48" s="2" t="inlineStr">
@@ -5664,7 +5664,7 @@
       </c>
       <c r="AD49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE49" s="2" t="inlineStr">
@@ -5766,7 +5766,7 @@
       </c>
       <c r="AD50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE50" s="2" t="inlineStr">
@@ -5872,7 +5872,7 @@
       </c>
       <c r="AD51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE51" s="2" t="inlineStr">
@@ -5974,7 +5974,7 @@
       </c>
       <c r="AD52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE52" s="2" t="inlineStr">
@@ -6076,7 +6076,7 @@
       </c>
       <c r="AD53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE53" s="2" t="inlineStr">
@@ -6178,7 +6178,7 @@
       </c>
       <c r="AD54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE54" s="2" t="inlineStr">
@@ -6284,7 +6284,7 @@
       </c>
       <c r="AD55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE55" s="2" t="inlineStr">
@@ -6390,7 +6390,7 @@
       </c>
       <c r="AD56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE56" s="2" t="inlineStr">
@@ -6496,7 +6496,7 @@
       </c>
       <c r="AD57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE57" s="2" t="inlineStr">
@@ -6602,7 +6602,7 @@
       </c>
       <c r="AD58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE58" s="2" t="inlineStr">
@@ -6704,7 +6704,7 @@
       </c>
       <c r="AD59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE59" s="2" t="inlineStr">
@@ -6818,7 +6818,7 @@
       </c>
       <c r="AD60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE60" s="2" t="inlineStr">
@@ -6920,7 +6920,7 @@
       </c>
       <c r="AD61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE61" s="2" t="inlineStr">
@@ -7034,7 +7034,7 @@
       </c>
       <c r="AD62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE62" s="2" t="inlineStr">
@@ -7140,7 +7140,7 @@
       </c>
       <c r="AD63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE63" s="2" t="inlineStr">
@@ -7246,7 +7246,7 @@
       </c>
       <c r="AD64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE64" s="2" t="inlineStr">
@@ -7352,7 +7352,7 @@
       </c>
       <c r="AD65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE65" s="2" t="inlineStr">
@@ -7458,7 +7458,7 @@
       </c>
       <c r="AD66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE66" s="2" t="inlineStr">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="AD67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE67" s="2" t="inlineStr">
@@ -7670,7 +7670,7 @@
       </c>
       <c r="AD68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE68" s="2" t="inlineStr">
@@ -7772,7 +7772,7 @@
       </c>
       <c r="AD69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE69" s="2" t="inlineStr">
@@ -7874,7 +7874,7 @@
       </c>
       <c r="AD70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE70" s="2" t="inlineStr">
@@ -7976,7 +7976,7 @@
       </c>
       <c r="AD71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE71" s="2" t="inlineStr">
@@ -8078,7 +8078,7 @@
       </c>
       <c r="AD72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE72" s="2" t="inlineStr">
@@ -8180,7 +8180,7 @@
       </c>
       <c r="AD73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE73" s="2" t="inlineStr">
@@ -8286,7 +8286,7 @@
       </c>
       <c r="AD74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE74" s="2" t="inlineStr">
@@ -8392,7 +8392,7 @@
       </c>
       <c r="AD75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE75" s="2" t="inlineStr">
@@ -8498,7 +8498,7 @@
       </c>
       <c r="AD76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE76" s="2" t="inlineStr">
@@ -8604,7 +8604,7 @@
       </c>
       <c r="AD77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE77" s="2" t="inlineStr">
@@ -8710,7 +8710,7 @@
       </c>
       <c r="AD78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE78" s="2" t="inlineStr">
@@ -8816,7 +8816,7 @@
       </c>
       <c r="AD79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE79" s="2" t="inlineStr">
@@ -8922,7 +8922,7 @@
       </c>
       <c r="AD80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE80" s="2" t="inlineStr">
@@ -9028,7 +9028,7 @@
       </c>
       <c r="AD81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE81" s="2" t="inlineStr">
@@ -9134,7 +9134,7 @@
       </c>
       <c r="AD82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE82" s="2" t="inlineStr">
@@ -9240,7 +9240,7 @@
       </c>
       <c r="AD83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE83" s="2" t="inlineStr">
@@ -9346,7 +9346,7 @@
       </c>
       <c r="AD84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE84" s="2" t="inlineStr">
@@ -9448,7 +9448,7 @@
       </c>
       <c r="AD85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE85" s="2" t="inlineStr">
@@ -9554,7 +9554,7 @@
       </c>
       <c r="AD86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE86" s="2" t="inlineStr">
@@ -9660,7 +9660,7 @@
       </c>
       <c r="AD87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE87" s="2" t="inlineStr">
@@ -9766,7 +9766,7 @@
       </c>
       <c r="AD88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE88" s="2" t="inlineStr">
@@ -9872,7 +9872,7 @@
       </c>
       <c r="AD89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE89" s="2" t="inlineStr">
@@ -9978,7 +9978,7 @@
       </c>
       <c r="AD90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE90" s="2" t="inlineStr">
@@ -10084,7 +10084,7 @@
       </c>
       <c r="AD91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE91" s="2" t="inlineStr">
@@ -10190,7 +10190,7 @@
       </c>
       <c r="AD92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE92" s="2" t="inlineStr">
@@ -10296,7 +10296,7 @@
       </c>
       <c r="AD93" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE93" s="2" t="inlineStr">
@@ -10402,7 +10402,7 @@
       </c>
       <c r="AD94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE94" s="2" t="inlineStr">
@@ -10504,7 +10504,7 @@
       </c>
       <c r="AD95" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE95" s="2" t="inlineStr">
@@ -10606,7 +10606,7 @@
       </c>
       <c r="AD96" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE96" s="2" t="inlineStr">
@@ -10708,7 +10708,7 @@
       </c>
       <c r="AD97" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE97" s="2" t="inlineStr">
@@ -10810,7 +10810,7 @@
       </c>
       <c r="AD98" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE98" s="2" t="inlineStr">
@@ -10912,7 +10912,7 @@
       </c>
       <c r="AD99" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE99" s="2" t="inlineStr">
@@ -11014,7 +11014,7 @@
       </c>
       <c r="AD100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE100" s="2" t="inlineStr">
@@ -11116,7 +11116,7 @@
       </c>
       <c r="AD101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE101" s="2" t="inlineStr">
@@ -11218,7 +11218,7 @@
       </c>
       <c r="AD102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE102" s="2" t="inlineStr">
@@ -11320,7 +11320,7 @@
       </c>
       <c r="AD103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE103" s="2" t="inlineStr">
@@ -11422,7 +11422,7 @@
       </c>
       <c r="AD104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE104" s="2" t="inlineStr">
@@ -11524,7 +11524,7 @@
       </c>
       <c r="AD105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE105" s="2" t="inlineStr">
@@ -11626,7 +11626,7 @@
       </c>
       <c r="AD106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE106" s="2" t="inlineStr">
@@ -11728,7 +11728,7 @@
       </c>
       <c r="AD107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE107" s="2" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="AD108" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE108" s="2" t="inlineStr">
@@ -11932,7 +11932,7 @@
       </c>
       <c r="AD109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE109" s="2" t="inlineStr">
@@ -12034,7 +12034,7 @@
       </c>
       <c r="AD110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE110" s="2" t="inlineStr">
@@ -12136,7 +12136,7 @@
       </c>
       <c r="AD111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE111" s="2" t="inlineStr">
@@ -12234,7 +12234,7 @@
       </c>
       <c r="AD112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE112" s="2" t="inlineStr">
@@ -12332,7 +12332,7 @@
       </c>
       <c r="AD113" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE113" s="2" t="inlineStr">
@@ -12430,7 +12430,7 @@
       </c>
       <c r="AD114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE114" s="2" t="inlineStr">
@@ -12528,7 +12528,7 @@
       </c>
       <c r="AD115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE115" s="2" t="inlineStr">
@@ -12626,7 +12626,7 @@
       </c>
       <c r="AD116" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE116" s="2" t="inlineStr">
@@ -12724,7 +12724,7 @@
       </c>
       <c r="AD117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE117" s="2" t="inlineStr">
@@ -12822,7 +12822,7 @@
       </c>
       <c r="AD118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE118" s="2" t="inlineStr">
@@ -12920,7 +12920,7 @@
       </c>
       <c r="AD119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE119" s="2" t="inlineStr">
@@ -13018,7 +13018,7 @@
       </c>
       <c r="AD120" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE120" s="2" t="inlineStr">
@@ -13116,7 +13116,7 @@
       </c>
       <c r="AD121" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE121" s="2" t="inlineStr">
@@ -13218,7 +13218,7 @@
       </c>
       <c r="AD122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE122" s="2" t="inlineStr">
@@ -13320,7 +13320,7 @@
       </c>
       <c r="AD123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE123" s="2" t="inlineStr">
@@ -13422,7 +13422,7 @@
       </c>
       <c r="AD124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE124" s="2" t="inlineStr">
@@ -13524,7 +13524,7 @@
       </c>
       <c r="AD125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE125" s="2" t="inlineStr">
@@ -13626,7 +13626,7 @@
       </c>
       <c r="AD126" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE126" s="2" t="inlineStr">
@@ -13724,7 +13724,7 @@
       </c>
       <c r="AD127" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE127" s="2" t="inlineStr">
@@ -13826,7 +13826,7 @@
       </c>
       <c r="AD128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE128" s="2" t="inlineStr">
@@ -13924,7 +13924,7 @@
       </c>
       <c r="AD129" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE129" s="2" t="inlineStr">
@@ -14022,7 +14022,7 @@
       </c>
       <c r="AD130" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE130" s="2" t="inlineStr">
@@ -14120,7 +14120,7 @@
       </c>
       <c r="AD131" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE131" s="2" t="inlineStr">
@@ -14222,7 +14222,7 @@
       </c>
       <c r="AD132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE132" s="2" t="inlineStr">
@@ -14320,7 +14320,7 @@
       </c>
       <c r="AD133" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE133" s="2" t="inlineStr">
@@ -14418,7 +14418,7 @@
       </c>
       <c r="AD134" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE134" s="2" t="inlineStr">
@@ -14520,7 +14520,7 @@
       </c>
       <c r="AD135" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE135" s="2" t="inlineStr">
@@ -14618,7 +14618,7 @@
       </c>
       <c r="AD136" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE136" s="2" t="inlineStr">
@@ -14720,7 +14720,7 @@
       </c>
       <c r="AD137" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE137" s="2" t="inlineStr">
@@ -14822,7 +14822,7 @@
       </c>
       <c r="AD138" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE138" s="2" t="inlineStr">
@@ -14924,7 +14924,7 @@
       </c>
       <c r="AD139" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE139" s="2" t="inlineStr">
@@ -15022,7 +15022,7 @@
       </c>
       <c r="AD140" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE140" s="2" t="inlineStr">
@@ -15120,7 +15120,7 @@
       </c>
       <c r="AD141" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE141" s="2" t="inlineStr">
@@ -15218,7 +15218,7 @@
       </c>
       <c r="AD142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE142" s="2" t="inlineStr">
@@ -15316,7 +15316,7 @@
       </c>
       <c r="AD143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE143" s="2" t="inlineStr">
@@ -15414,7 +15414,7 @@
       </c>
       <c r="AD144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE144" s="2" t="inlineStr">
@@ -15512,7 +15512,7 @@
       </c>
       <c r="AD145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE145" s="2" t="inlineStr">
@@ -15610,7 +15610,7 @@
       </c>
       <c r="AD146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE146" s="2" t="inlineStr">
@@ -15708,7 +15708,7 @@
       </c>
       <c r="AD147" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE147" s="2" t="inlineStr">
@@ -15806,7 +15806,7 @@
       </c>
       <c r="AD148" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE148" s="2" t="inlineStr">
@@ -15904,7 +15904,7 @@
       </c>
       <c r="AD149" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE149" s="2" t="inlineStr">
@@ -16002,7 +16002,7 @@
       </c>
       <c r="AD150" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE150" s="2" t="inlineStr">
@@ -16100,7 +16100,7 @@
       </c>
       <c r="AD151" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE151" s="2" t="inlineStr">
@@ -16198,7 +16198,7 @@
       </c>
       <c r="AD152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE152" s="2" t="inlineStr">
@@ -16296,7 +16296,7 @@
       </c>
       <c r="AD153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE153" s="2" t="inlineStr">
@@ -16394,7 +16394,7 @@
       </c>
       <c r="AD154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE154" s="2" t="inlineStr">
@@ -16492,7 +16492,7 @@
       </c>
       <c r="AD155" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE155" s="2" t="inlineStr">
@@ -16590,7 +16590,7 @@
       </c>
       <c r="AD156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE156" s="2" t="inlineStr">
@@ -16688,7 +16688,7 @@
       </c>
       <c r="AD157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE157" s="2" t="inlineStr">
@@ -16786,7 +16786,7 @@
       </c>
       <c r="AD158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE158" s="2" t="inlineStr">
@@ -16884,7 +16884,7 @@
       </c>
       <c r="AD159" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE159" s="2" t="inlineStr">
@@ -16982,7 +16982,7 @@
       </c>
       <c r="AD160" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE160" s="2" t="inlineStr">
@@ -17080,7 +17080,7 @@
       </c>
       <c r="AD161" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE161" s="2" t="inlineStr">
@@ -17178,7 +17178,7 @@
       </c>
       <c r="AD162" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE162" s="2" t="inlineStr">
@@ -17276,7 +17276,7 @@
       </c>
       <c r="AD163" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE163" s="2" t="inlineStr">
@@ -17374,7 +17374,7 @@
       </c>
       <c r="AD164" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37</t>
+          <t>2026-10-31 19:30</t>
         </is>
       </c>
       <c r="AE164" s="2" t="inlineStr">
@@ -17443,7 +17443,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37 UTC</t>
+          <t>2026-10-31 19:30 UTC</t>
         </is>
       </c>
     </row>
@@ -17455,7 +17455,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-31 13:37 UTC</t>
+          <t>2026-10-31 19:31 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>